<commit_message>
added TC_09 and TC_10
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestOutput.xlsx
+++ b/src/test/resources/testdata/TestOutput.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="18">
   <si>
     <t>S.No</t>
   </si>
@@ -66,6 +66,15 @@
   </si>
   <si>
     <t>Dining Room</t>
+  </si>
+  <si>
+    <t>TC_10 - Product Image URL</t>
+  </si>
+  <si>
+    <t>Image URL</t>
+  </si>
+  <si>
+    <t>https://cdn.swadeshonline.com/v2/patient-paper-41f385/swad-p/wrkr/products/pictures/item/free/450x0/PQc-XAw0n-a.jpg</t>
   </si>
 </sst>
 </file>
@@ -438,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -549,6 +558,36 @@
       </c>
       <c r="C10" t="s" s="0">
         <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed xpath and linespaces
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestOutput.xlsx
+++ b/src/test/resources/testdata/TestOutput.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="46">
   <si>
     <t>S.No</t>
   </si>
@@ -1271,7 +1271,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4018DD7B-01A5-4810-8DB3-FB76076E4E02}">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="19.0"/>
@@ -1477,6 +1477,46 @@
         <v>14</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated automation framework and test cases
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestOutput.xlsx
+++ b/src/test/resources/testdata/TestOutput.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="58">
   <si>
     <t>S.No</t>
   </si>
@@ -187,6 +187,15 @@
   </si>
   <si>
     <t>Cabalo Solid Wood Dining Chair in Dark Walnut Finish - Set of 2</t>
+  </si>
+  <si>
+    <t>₹9,599</t>
+  </si>
+  <si>
+    <t>Rhodes Solid Wood Bookshelf in Teak Finish</t>
+  </si>
+  <si>
+    <t>₹9,999</t>
   </si>
 </sst>
 </file>
@@ -559,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C209"/>
+  <dimension ref="A1:C241"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -2542,6 +2551,290 @@
     </row>
     <row r="209">
       <c r="A209" t="s" s="0">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n" s="0">
+        <v>209.0</v>
+      </c>
+      <c r="B210" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C210" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n" s="0">
+        <v>210.0</v>
+      </c>
+      <c r="B211" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C211" t="s" s="0">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n" s="0">
+        <v>211.0</v>
+      </c>
+      <c r="B212" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="C212" t="s" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B216" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C216" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B217" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C217" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B218" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C218" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B219" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C219" t="s" s="0">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B220" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C220" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B221" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C221" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="B222" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C222" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="B223" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C223" t="s" s="0">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="B224" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="C224" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="B225" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C225" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="B226" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C226" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="B227" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C227" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="B228" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C228" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="B229" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C229" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n" s="0">
+        <v>14.0</v>
+      </c>
+      <c r="B230" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C230" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="B231" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C231" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n" s="0">
+        <v>16.0</v>
+      </c>
+      <c r="B232" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C232" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n" s="0">
+        <v>17.0</v>
+      </c>
+      <c r="B233" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C233" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n" s="0">
+        <v>18.0</v>
+      </c>
+      <c r="B234" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C234" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="B235" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C235" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="B236" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C236" t="s" s="0">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="s" s="0">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="s" s="0">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="s" s="0">
         <v>51</v>
       </c>
     </row>
@@ -2552,7 +2845,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4018DD7B-01A5-4810-8DB3-FB76076E4E02}">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="19.0"/>
@@ -2798,6 +3091,86 @@
         <v>14</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2805,7 +3178,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2880,6 +3253,30 @@
         <v>54</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>54</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>